<commit_message>
begin ov avk pravki
</commit_message>
<xml_diff>
--- a/burocracy/diss_council.xlsx
+++ b/burocracy/diss_council.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\PhD\disser\burocracy\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7FA6EA4C-D3E0-420D-BD0E-D07E061A75C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E27401A1-6EE4-43E1-938A-6F5C0D851376}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{134430FC-25E2-4572-9815-FE2A91FBD179}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="71">
   <si>
     <t>№</t>
   </si>
@@ -132,9 +132,6 @@
     <t>председатель</t>
   </si>
   <si>
-    <t>точно будет</t>
-  </si>
-  <si>
     <t>Кузнецов</t>
   </si>
   <si>
@@ -216,17 +213,48 @@
     <t>Мещеринов Вячеслав Вячеславович</t>
   </si>
   <si>
-    <t>Написал рыбу?</t>
-  </si>
-  <si>
     <t>Да</t>
+  </si>
+  <si>
+    <t>Контакты</t>
+  </si>
+  <si>
+    <t>Написал рыбу анкеты?</t>
+  </si>
+  <si>
+    <t>astval@mail.ru
+astapenko.va@phystech.edu
+8(962)993-89-04</t>
+  </si>
+  <si>
+    <t>Председатель</t>
+  </si>
+  <si>
+    <t>8 (495) 702-93-17
+nailinogamov@gmail.com</t>
+  </si>
+  <si>
+    <t>vpkrainov@mail.ru
+krainov.vp@phystech.edu</t>
+  </si>
+  <si>
+    <t>kudryashovsi@lebedev.ru
+8(499) 132-60-83
+8(903) 185-02-46</t>
+  </si>
+  <si>
+    <t>8 903 504 9852
+murzina@mail.ru</t>
+  </si>
+  <si>
+    <t>vitukhnovsky@mail.ru +7(499) 132-63-64</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -235,8 +263,24 @@
       <charset val="204"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="204"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+      <charset val="204"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -245,18 +289,24 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
+        <fgColor theme="7" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.59999389629810485"/>
+        <fgColor theme="4" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.14999847407452621"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -264,16 +314,51 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Гиперссылка" xfId="1" builtinId="8"/>
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -586,7 +671,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A3A0C460-2CFB-4414-A3CC-DFB3884CADAE}">
-  <dimension ref="A1:K14"/>
+  <dimension ref="A1:M14"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14" bestFit="1" customWidth="1"/>
@@ -596,345 +681,437 @@
     <col min="6" max="6" width="9.88671875" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="47.88671875" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="27.44140625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="11.77734375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="27.44140625" customWidth="1"/>
+    <col min="10" max="10" width="11.77734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
+        <v>63</v>
+      </c>
+      <c r="L1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A2" s="4"/>
+      <c r="B2" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="F2" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="G2" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="H2" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="I2" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="K1" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="B2" t="s">
-        <v>0</v>
-      </c>
-      <c r="C2" t="s">
+      <c r="J2" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="K2" s="4"/>
+      <c r="L2" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="M2" s="4"/>
+    </row>
+    <row r="3" spans="1:13" s="2" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A3" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="B3" s="5">
+        <v>1</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="F3" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="G3" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="H3" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="I3" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="J3" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="K3" s="5"/>
+      <c r="L3" s="5"/>
+      <c r="M3" s="5"/>
+    </row>
+    <row r="4" spans="1:13" s="2" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A4" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="B4" s="5">
         <v>2</v>
       </c>
-      <c r="D2" t="s">
-        <v>1</v>
-      </c>
-      <c r="E2" t="s">
+      <c r="C4" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="H4" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="I4" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="J4" s="5"/>
+      <c r="K4" s="5"/>
+      <c r="L4" s="5"/>
+      <c r="M4" s="5"/>
+    </row>
+    <row r="5" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="B5" s="5">
         <v>3</v>
       </c>
-      <c r="F2" t="s">
+      <c r="C5" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="H5" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="I5" s="7" t="s">
+        <v>70</v>
+      </c>
+      <c r="J5" s="5"/>
+      <c r="K5" s="5"/>
+      <c r="L5" s="5"/>
+      <c r="M5" s="5"/>
+    </row>
+    <row r="6" spans="1:13" s="1" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A6" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="B6" s="8">
+        <v>4</v>
+      </c>
+      <c r="C6" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="D6" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="E6" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="F6" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="G6" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="H6" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="I6" s="9" t="s">
+        <v>68</v>
+      </c>
+      <c r="J6" s="8"/>
+      <c r="K6" s="8"/>
+      <c r="L6" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="M6" s="8"/>
+    </row>
+    <row r="7" spans="1:13" s="1" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A7" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="B7" s="8">
+        <v>5</v>
+      </c>
+      <c r="C7" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="D7" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="E7" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="F7" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="G7" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="H7" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="I7" s="10" t="s">
+        <v>69</v>
+      </c>
+      <c r="J7" s="8"/>
+      <c r="K7" s="8"/>
+      <c r="L7" s="8"/>
+      <c r="M7" s="8"/>
+    </row>
+    <row r="8" spans="1:13" s="1" customFormat="1" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="A8" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="B8" s="8">
+        <v>6</v>
+      </c>
+      <c r="C8" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="D8" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="E8" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="F8" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="G8" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="H8" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="I8" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="J8" s="8"/>
+      <c r="K8" s="8"/>
+      <c r="L8" s="8"/>
+      <c r="M8" s="8"/>
+    </row>
+    <row r="9" spans="1:13" s="3" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="12"/>
+      <c r="B9" s="12">
+        <v>7</v>
+      </c>
+      <c r="C9" s="12" t="s">
+        <v>53</v>
+      </c>
+      <c r="D9" s="12" t="s">
+        <v>54</v>
+      </c>
+      <c r="E9" s="12" t="s">
+        <v>36</v>
+      </c>
+      <c r="F9" s="12" t="s">
+        <v>10</v>
+      </c>
+      <c r="G9" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="H9" s="12" t="s">
+        <v>55</v>
+      </c>
+      <c r="I9" s="12"/>
+      <c r="J9" s="12"/>
+      <c r="K9" s="12"/>
+      <c r="L9" s="12"/>
+      <c r="M9" s="12"/>
+    </row>
+    <row r="10" spans="1:13" s="3" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="12"/>
+      <c r="B10" s="12">
+        <v>8</v>
+      </c>
+      <c r="C10" s="12" t="s">
+        <v>56</v>
+      </c>
+      <c r="D10" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="E10" s="12" t="s">
+        <v>58</v>
+      </c>
+      <c r="F10" s="12" t="s">
+        <v>10</v>
+      </c>
+      <c r="G10" s="12" t="s">
+        <v>59</v>
+      </c>
+      <c r="H10" s="12" t="s">
+        <v>60</v>
+      </c>
+      <c r="I10" s="12"/>
+      <c r="J10" s="12"/>
+      <c r="K10" s="12"/>
+      <c r="L10" s="12"/>
+      <c r="M10" s="12"/>
+    </row>
+    <row r="11" spans="1:13" s="3" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="12"/>
+      <c r="B11" s="12">
         <v>9</v>
       </c>
-      <c r="G2" t="s">
-        <v>4</v>
-      </c>
-      <c r="H2" t="s">
-        <v>5</v>
-      </c>
-      <c r="I2" t="s">
-        <v>29</v>
-      </c>
-      <c r="K2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="B3" s="2">
-        <v>1</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="F3" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="G3" s="2" t="s">
+      <c r="C11" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="D11" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="E11" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="F11" s="12" t="s">
+        <v>10</v>
+      </c>
+      <c r="G11" s="12" t="s">
         <v>20</v>
       </c>
-      <c r="H3" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="I3" s="2" t="s">
+      <c r="H11" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="I11" s="12"/>
+      <c r="J11" s="12"/>
+      <c r="K11" s="12"/>
+      <c r="L11" s="12"/>
+      <c r="M11" s="12"/>
+    </row>
+    <row r="12" spans="1:13" s="3" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="12"/>
+      <c r="B12" s="12">
+        <v>10</v>
+      </c>
+      <c r="C12" s="12" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="4" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="B4" s="1">
-        <v>2</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="E4" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="F4" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="G4" s="1" t="s">
+      <c r="D12" s="12" t="s">
+        <v>35</v>
+      </c>
+      <c r="E12" s="12" t="s">
+        <v>36</v>
+      </c>
+      <c r="F12" s="12" t="s">
+        <v>10</v>
+      </c>
+      <c r="G12" s="12" t="s">
+        <v>37</v>
+      </c>
+      <c r="H12" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="I12" s="12"/>
+      <c r="J12" s="12"/>
+      <c r="K12" s="12"/>
+      <c r="L12" s="12"/>
+      <c r="M12" s="12"/>
+    </row>
+    <row r="13" spans="1:13" s="3" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="12"/>
+      <c r="B13" s="12">
         <v>11</v>
       </c>
-      <c r="H4" s="1" t="s">
+      <c r="C13" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="D13" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="E13" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="F13" s="12" t="s">
+        <v>10</v>
+      </c>
+      <c r="G13" s="12" t="s">
+        <v>41</v>
+      </c>
+      <c r="H13" s="12" t="s">
+        <v>42</v>
+      </c>
+      <c r="I13" s="12"/>
+      <c r="J13" s="12"/>
+      <c r="K13" s="12"/>
+      <c r="L13" s="12"/>
+      <c r="M13" s="12"/>
+    </row>
+    <row r="14" spans="1:13" s="3" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="12"/>
+      <c r="B14" s="12">
         <v>12</v>
       </c>
-      <c r="K4" s="1" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="B5" s="1">
-        <v>3</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="E5" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="F5" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="G5" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="H5" s="1" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="B6">
-        <v>4</v>
-      </c>
-      <c r="C6" t="s">
-        <v>17</v>
-      </c>
-      <c r="D6" t="s">
-        <v>18</v>
-      </c>
-      <c r="E6" t="s">
-        <v>19</v>
-      </c>
-      <c r="F6" t="s">
-        <v>10</v>
-      </c>
-      <c r="G6" t="s">
-        <v>20</v>
-      </c>
-      <c r="H6" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="B7" s="1">
-        <v>5</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="E7" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="F7" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="G7" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="H7" s="1" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="B8">
-        <v>6</v>
-      </c>
-      <c r="C8" t="s">
-        <v>35</v>
-      </c>
-      <c r="D8" t="s">
-        <v>36</v>
-      </c>
-      <c r="E8" t="s">
-        <v>37</v>
-      </c>
-      <c r="F8" t="s">
-        <v>10</v>
-      </c>
-      <c r="G8" t="s">
-        <v>38</v>
-      </c>
-      <c r="H8" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="B9">
-        <v>7</v>
-      </c>
-      <c r="C9" t="s">
-        <v>39</v>
-      </c>
-      <c r="D9" t="s">
-        <v>40</v>
-      </c>
-      <c r="E9" t="s">
-        <v>41</v>
-      </c>
-      <c r="F9" t="s">
-        <v>10</v>
-      </c>
-      <c r="G9" t="s">
-        <v>42</v>
-      </c>
-      <c r="H9" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="10" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="B10" s="2">
-        <v>8</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="D10" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="E10" s="2" t="s">
+      <c r="C14" s="12" t="s">
         <v>46</v>
       </c>
-      <c r="F10" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="G10" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="H10" s="2" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="B11">
-        <v>9</v>
-      </c>
-      <c r="C11" t="s">
+      <c r="D14" s="12" t="s">
         <v>47</v>
       </c>
-      <c r="D11" t="s">
+      <c r="E14" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="E11" t="s">
+      <c r="F14" s="12" t="s">
+        <v>10</v>
+      </c>
+      <c r="G14" s="12" t="s">
         <v>49</v>
       </c>
-      <c r="F11" t="s">
-        <v>10</v>
-      </c>
-      <c r="G11" t="s">
+      <c r="H14" s="12" t="s">
         <v>50</v>
       </c>
-      <c r="H11" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="12" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="B12" s="2">
-        <v>10</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="D12" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="E12" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="F12" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="G12" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="H12" s="2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="B13">
-        <v>11</v>
-      </c>
-      <c r="C13" t="s">
-        <v>54</v>
-      </c>
-      <c r="D13" t="s">
-        <v>55</v>
-      </c>
-      <c r="E13" t="s">
-        <v>37</v>
-      </c>
-      <c r="F13" t="s">
-        <v>10</v>
-      </c>
-      <c r="G13" t="s">
-        <v>20</v>
-      </c>
-      <c r="H13" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="B14">
-        <v>12</v>
-      </c>
-      <c r="C14" t="s">
-        <v>57</v>
-      </c>
-      <c r="D14" t="s">
-        <v>58</v>
-      </c>
-      <c r="E14" t="s">
-        <v>59</v>
-      </c>
-      <c r="F14" t="s">
-        <v>10</v>
-      </c>
-      <c r="G14" t="s">
-        <v>60</v>
-      </c>
-      <c r="H14" t="s">
-        <v>61</v>
-      </c>
+      <c r="I14" s="12"/>
+      <c r="J14" s="12"/>
+      <c r="K14" s="12"/>
+      <c r="L14" s="12"/>
+      <c r="M14" s="12"/>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="I3" r:id="rId1" display="astval@mail.ru_x000a_8(962)993-89-04" xr:uid="{55B80AD8-BB63-400C-82C8-D1A2D95E682B}"/>
+    <hyperlink ref="I4" r:id="rId2" display="mailto:vpkrainov@mail.ru" xr:uid="{B85A9B67-6B35-4E7E-B7BA-C6FE4984F297}"/>
+    <hyperlink ref="I6" r:id="rId3" xr:uid="{1B5ADA78-8CBD-43E8-A167-CE865E1C4D3A}"/>
+    <hyperlink ref="I5" r:id="rId4" display="mailto:vitukhnovsky@mail.ru" xr:uid="{A2FFBEB8-9E0D-469A-A860-49F874F54EBF}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
new dc data add
</commit_message>
<xml_diff>
--- a/burocracy/diss_council.xlsx
+++ b/burocracy/diss_council.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\PhD\disser\burocracy\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9D122B2-BC82-4CB2-9961-74C79E4A0905}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BEDBF539-A84F-4E57-B77E-042444C7B5BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{134430FC-25E2-4572-9815-FE2A91FBD179}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="91">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="145" uniqueCount="97">
   <si>
     <t>Имя</t>
   </si>
@@ -308,6 +308,24 @@
   </si>
   <si>
     <t>Написал 19 августа</t>
+  </si>
+  <si>
+    <t>Макаров</t>
+  </si>
+  <si>
+    <t>Дмитрий</t>
+  </si>
+  <si>
+    <t>Северный институт</t>
+  </si>
+  <si>
+    <t>d.makarov@narfu.ru</t>
+  </si>
+  <si>
+    <t>только онлайн</t>
+  </si>
+  <si>
+    <t>может не хватить публикаций</t>
   </si>
 </sst>
 </file>
@@ -770,7 +788,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A3A0C460-2CFB-4414-A3CC-DFB3884CADAE}">
-  <dimension ref="A1:O17"/>
+  <dimension ref="A1:O18"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14" style="5" bestFit="1" customWidth="1"/>
@@ -913,7 +931,7 @@
       <c r="N4" s="7"/>
       <c r="O4" s="7"/>
     </row>
-    <row r="5" spans="1:15" s="8" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:15" s="8" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A5" s="7" t="s">
         <v>60</v>
       </c>
@@ -945,47 +963,51 @@
       <c r="K5" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="L5" s="7"/>
+      <c r="L5" s="7" t="s">
+        <v>96</v>
+      </c>
       <c r="M5" s="7"/>
       <c r="N5" s="7"/>
       <c r="O5" s="7"/>
     </row>
-    <row r="6" spans="1:15" s="8" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A6" s="7" t="s">
-        <v>60</v>
-      </c>
-      <c r="B6" s="7" t="s">
-        <v>73</v>
-      </c>
-      <c r="C6" s="7"/>
-      <c r="D6" s="7"/>
-      <c r="E6" s="7" t="s">
-        <v>50</v>
-      </c>
-      <c r="F6" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="G6" s="7" t="s">
-        <v>51</v>
-      </c>
-      <c r="H6" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="I6" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="J6" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="K6" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="L6" s="7"/>
-      <c r="M6" s="7"/>
-      <c r="N6" s="7"/>
-      <c r="O6" s="7"/>
-    </row>
-    <row r="7" spans="1:15" s="11" customFormat="1" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:15" s="11" customFormat="1" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="A6" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="D6" s="2"/>
+      <c r="E6" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="H6" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="I6" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="J6" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K6" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="L6" s="2"/>
+      <c r="M6" s="2"/>
+      <c r="N6" s="2"/>
+      <c r="O6" s="2"/>
+    </row>
+    <row r="7" spans="1:15" s="11" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
         <v>60</v>
       </c>
@@ -997,224 +1019,232 @@
       </c>
       <c r="D7" s="2"/>
       <c r="E7" s="2" t="s">
-        <v>21</v>
+        <v>91</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>22</v>
+        <v>92</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>23</v>
+        <v>87</v>
       </c>
       <c r="H7" s="2" t="s">
         <v>9</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>27</v>
+        <v>93</v>
       </c>
       <c r="J7" s="2" t="s">
-        <v>20</v>
+        <v>81</v>
       </c>
       <c r="K7" s="3" t="s">
-        <v>65</v>
-      </c>
-      <c r="L7" s="2"/>
+        <v>94</v>
+      </c>
+      <c r="L7" s="2" t="s">
+        <v>95</v>
+      </c>
       <c r="M7" s="2"/>
       <c r="N7" s="2"/>
       <c r="O7" s="2"/>
     </row>
-    <row r="8" spans="1:15" s="11" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="2" t="s">
+    <row r="8" spans="1:15" s="8" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A8" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>73</v>
+      </c>
+      <c r="C8" s="7"/>
+      <c r="D8" s="7"/>
+      <c r="E8" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="F8" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="G8" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="H8" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="I8" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="J8" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="K8" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="L8" s="7"/>
+      <c r="M8" s="7"/>
+      <c r="N8" s="7"/>
+      <c r="O8" s="7"/>
+    </row>
+    <row r="9" spans="1:15" s="11" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="B9" s="2" t="s">
         <v>76</v>
-      </c>
-      <c r="C8" s="2"/>
-      <c r="D8" s="2"/>
-      <c r="E8" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="F8" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="G8" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="H8" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="I8" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="J8" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="K8" s="14" t="s">
-        <v>77</v>
-      </c>
-      <c r="L8" s="2"/>
-      <c r="M8" s="2"/>
-      <c r="N8" s="2"/>
-      <c r="O8" s="2"/>
-    </row>
-    <row r="9" spans="1:15" s="11" customFormat="1" ht="32.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>84</v>
       </c>
       <c r="C9" s="2"/>
       <c r="D9" s="2"/>
       <c r="E9" s="2" t="s">
-        <v>12</v>
+        <v>33</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>13</v>
+        <v>34</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>14</v>
+        <v>35</v>
       </c>
       <c r="H9" s="2" t="s">
         <v>9</v>
       </c>
       <c r="I9" s="2" t="s">
-        <v>15</v>
+        <v>36</v>
       </c>
       <c r="J9" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="K9" s="2" t="s">
-        <v>68</v>
+        <v>20</v>
+      </c>
+      <c r="K9" s="14" t="s">
+        <v>77</v>
       </c>
       <c r="L9" s="2"/>
       <c r="M9" s="2"/>
       <c r="N9" s="2"/>
       <c r="O9" s="2"/>
     </row>
-    <row r="10" spans="1:15" s="8" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="7"/>
-      <c r="B10" s="7" t="s">
+    <row r="10" spans="1:15" s="11" customFormat="1" ht="32.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="C10" s="2"/>
+      <c r="D10" s="2"/>
+      <c r="E10" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G10" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H10" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="I10" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="J10" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="K10" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="L10" s="2"/>
+      <c r="M10" s="2"/>
+      <c r="N10" s="2"/>
+      <c r="O10" s="2"/>
+    </row>
+    <row r="11" spans="1:15" s="8" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="7"/>
+      <c r="B11" s="7" t="s">
         <v>83</v>
       </c>
-      <c r="C10" s="7"/>
-      <c r="D10" s="7"/>
-      <c r="E10" s="7" t="s">
+      <c r="C11" s="7"/>
+      <c r="D11" s="7"/>
+      <c r="E11" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="F10" s="7" t="s">
+      <c r="F11" s="7" t="s">
         <v>53</v>
       </c>
-      <c r="G10" s="7" t="s">
+      <c r="G11" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="H10" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="I10" s="7" t="s">
+      <c r="H11" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="I11" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="J10" s="7" t="s">
+      <c r="J11" s="7" t="s">
         <v>54</v>
       </c>
-      <c r="K10" s="7"/>
-      <c r="L10" s="7"/>
-      <c r="M10" s="7"/>
-      <c r="N10" s="7"/>
-      <c r="O10" s="7"/>
-    </row>
-    <row r="11" spans="1:15" s="11" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A11" s="2"/>
-      <c r="B11" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="C11" s="2"/>
-      <c r="D11" s="2"/>
-      <c r="E11" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="F11" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="G11" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="H11" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="I11" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="J11" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="K11" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="L11" s="2"/>
-      <c r="M11" s="2"/>
-      <c r="N11" s="2"/>
-      <c r="O11" s="2"/>
+      <c r="K11" s="7"/>
+      <c r="L11" s="7"/>
+      <c r="M11" s="7"/>
+      <c r="N11" s="7"/>
+      <c r="O11" s="7"/>
     </row>
     <row r="12" spans="1:15" s="11" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A12" s="2"/>
       <c r="B12" s="2" t="s">
-        <v>90</v>
+        <v>83</v>
       </c>
       <c r="C12" s="2"/>
       <c r="D12" s="2"/>
       <c r="E12" s="2" t="s">
-        <v>55</v>
+        <v>37</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>56</v>
+        <v>38</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>57</v>
+        <v>39</v>
       </c>
       <c r="H12" s="2" t="s">
         <v>9</v>
       </c>
       <c r="I12" s="2" t="s">
-        <v>58</v>
+        <v>40</v>
       </c>
       <c r="J12" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="K12" s="2"/>
+        <v>41</v>
+      </c>
+      <c r="K12" s="2" t="s">
+        <v>89</v>
+      </c>
       <c r="L12" s="2"/>
       <c r="M12" s="2"/>
       <c r="N12" s="2"/>
       <c r="O12" s="2"/>
     </row>
-    <row r="13" spans="1:15" s="10" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="9"/>
-      <c r="B13" s="9"/>
-      <c r="C13" s="9"/>
-      <c r="D13" s="9"/>
-      <c r="E13" s="9" t="s">
-        <v>16</v>
-      </c>
-      <c r="F13" s="9" t="s">
-        <v>17</v>
-      </c>
-      <c r="G13" s="9" t="s">
-        <v>18</v>
-      </c>
-      <c r="H13" s="9" t="s">
-        <v>9</v>
-      </c>
-      <c r="I13" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="J13" s="9" t="s">
-        <v>20</v>
-      </c>
-      <c r="K13" s="9"/>
-      <c r="L13" s="9"/>
-      <c r="M13" s="9"/>
-      <c r="N13" s="9"/>
-      <c r="O13" s="9"/>
+    <row r="13" spans="1:15" s="11" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A13" s="2"/>
+      <c r="B13" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="C13" s="2"/>
+      <c r="D13" s="2"/>
+      <c r="E13" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="F13" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="G13" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="H13" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="I13" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="J13" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="K13" s="2"/>
+      <c r="L13" s="2"/>
+      <c r="M13" s="2"/>
+      <c r="N13" s="2"/>
+      <c r="O13" s="2"/>
     </row>
     <row r="14" spans="1:15" s="10" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A14" s="9"/>
@@ -1222,22 +1252,22 @@
       <c r="C14" s="9"/>
       <c r="D14" s="9"/>
       <c r="E14" s="9" t="s">
-        <v>45</v>
+        <v>16</v>
       </c>
       <c r="F14" s="9" t="s">
-        <v>46</v>
+        <v>17</v>
       </c>
       <c r="G14" s="9" t="s">
-        <v>47</v>
+        <v>18</v>
       </c>
       <c r="H14" s="9" t="s">
         <v>9</v>
       </c>
       <c r="I14" s="9" t="s">
-        <v>48</v>
+        <v>19</v>
       </c>
       <c r="J14" s="9" t="s">
-        <v>49</v>
+        <v>20</v>
       </c>
       <c r="K14" s="9"/>
       <c r="L14" s="9"/>
@@ -1245,85 +1275,114 @@
       <c r="N14" s="9"/>
       <c r="O14" s="9"/>
     </row>
-    <row r="16" spans="1:15" s="13" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A16" s="12" t="s">
-        <v>60</v>
-      </c>
-      <c r="B16" s="12" t="s">
-        <v>74</v>
-      </c>
-      <c r="C16" s="12"/>
-      <c r="D16" s="12"/>
-      <c r="E16" s="12" t="s">
-        <v>5</v>
-      </c>
-      <c r="F16" s="12" t="s">
-        <v>6</v>
-      </c>
-      <c r="G16" s="12" t="s">
-        <v>7</v>
-      </c>
-      <c r="H16" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="I16" s="12" t="s">
-        <v>10</v>
-      </c>
-      <c r="J16" s="12" t="s">
-        <v>11</v>
-      </c>
-      <c r="K16" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="L16" s="12"/>
-      <c r="M16" s="12"/>
-      <c r="N16" s="12" t="s">
-        <v>26</v>
-      </c>
-      <c r="O16" s="12"/>
-    </row>
-    <row r="17" spans="1:15" s="13" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="12"/>
+    <row r="15" spans="1:15" s="10" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="9"/>
+      <c r="B15" s="9"/>
+      <c r="C15" s="9"/>
+      <c r="D15" s="9"/>
+      <c r="E15" s="9" t="s">
+        <v>45</v>
+      </c>
+      <c r="F15" s="9" t="s">
+        <v>46</v>
+      </c>
+      <c r="G15" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="H15" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="I15" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="J15" s="9" t="s">
+        <v>49</v>
+      </c>
+      <c r="K15" s="9"/>
+      <c r="L15" s="9"/>
+      <c r="M15" s="9"/>
+      <c r="N15" s="9"/>
+      <c r="O15" s="9"/>
+    </row>
+    <row r="17" spans="1:15" s="13" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A17" s="12" t="s">
+        <v>60</v>
+      </c>
       <c r="B17" s="12" t="s">
         <v>74</v>
       </c>
       <c r="C17" s="12"/>
       <c r="D17" s="12"/>
       <c r="E17" s="12" t="s">
-        <v>78</v>
+        <v>5</v>
       </c>
       <c r="F17" s="12" t="s">
-        <v>38</v>
+        <v>6</v>
       </c>
       <c r="G17" s="12" t="s">
-        <v>79</v>
+        <v>7</v>
       </c>
       <c r="H17" s="12" t="s">
         <v>9</v>
       </c>
       <c r="I17" s="12" t="s">
-        <v>80</v>
+        <v>10</v>
       </c>
       <c r="J17" s="12" t="s">
-        <v>81</v>
+        <v>11</v>
       </c>
       <c r="K17" s="4" t="s">
-        <v>82</v>
+        <v>67</v>
       </c>
       <c r="L17" s="12"/>
       <c r="M17" s="12"/>
-      <c r="N17" s="12"/>
+      <c r="N17" s="12" t="s">
+        <v>26</v>
+      </c>
       <c r="O17" s="12"/>
+    </row>
+    <row r="18" spans="1:15" s="13" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="12"/>
+      <c r="B18" s="12" t="s">
+        <v>74</v>
+      </c>
+      <c r="C18" s="12"/>
+      <c r="D18" s="12"/>
+      <c r="E18" s="12" t="s">
+        <v>78</v>
+      </c>
+      <c r="F18" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="G18" s="12" t="s">
+        <v>79</v>
+      </c>
+      <c r="H18" s="12" t="s">
+        <v>9</v>
+      </c>
+      <c r="I18" s="12" t="s">
+        <v>80</v>
+      </c>
+      <c r="J18" s="12" t="s">
+        <v>81</v>
+      </c>
+      <c r="K18" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="L18" s="12"/>
+      <c r="M18" s="12"/>
+      <c r="N18" s="12"/>
+      <c r="O18" s="12"/>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="K3" r:id="rId1" display="astval@mail.ru_x000a_8(962)993-89-04" xr:uid="{55B80AD8-BB63-400C-82C8-D1A2D95E682B}"/>
     <hyperlink ref="K4" r:id="rId2" display="mailto:vpkrainov@mail.ru" xr:uid="{B85A9B67-6B35-4E7E-B7BA-C6FE4984F297}"/>
-    <hyperlink ref="K16" r:id="rId3" xr:uid="{1B5ADA78-8CBD-43E8-A167-CE865E1C4D3A}"/>
-    <hyperlink ref="K6" r:id="rId4" display="mailto:vitukhnovsky@mail.ru" xr:uid="{A2FFBEB8-9E0D-469A-A860-49F874F54EBF}"/>
-    <hyperlink ref="K8" r:id="rId5" xr:uid="{4321ECF0-D9B7-4C17-8D2B-E91123E62F46}"/>
-    <hyperlink ref="K17" r:id="rId6" xr:uid="{1DF5DB8B-DE1C-4CE8-8E1F-37F1833ED1FE}"/>
-    <hyperlink ref="K5" r:id="rId7" xr:uid="{797371FE-0D11-42CE-8332-E27D72E9D370}"/>
+    <hyperlink ref="K17" r:id="rId3" xr:uid="{1B5ADA78-8CBD-43E8-A167-CE865E1C4D3A}"/>
+    <hyperlink ref="K9" r:id="rId4" xr:uid="{4321ECF0-D9B7-4C17-8D2B-E91123E62F46}"/>
+    <hyperlink ref="K18" r:id="rId5" xr:uid="{1DF5DB8B-DE1C-4CE8-8E1F-37F1833ED1FE}"/>
+    <hyperlink ref="K5" r:id="rId6" xr:uid="{797371FE-0D11-42CE-8332-E27D72E9D370}"/>
+    <hyperlink ref="K8" r:id="rId7" display="mailto:vitukhnovsky@mail.ru" xr:uid="{6DD08A79-9682-486A-8C22-FF1C2B887D81}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId8"/>

</xml_diff>